<commit_message>
Update PDS public dashboard/state: signal 2026-07, holding through 2026-08
</commit_message>
<xml_diff>
--- a/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
+++ b/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
@@ -25524,25 +25524,25 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.09578118377923987</v>
+        <v>0.09578120863437674</v>
       </c>
       <c r="E2" s="1">
-        <v>0.04522043298929932</v>
+        <v>0.04522044472396376</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
       </c>
       <c r="G2" s="1">
-        <v>0.02584024742245676</v>
+        <v>0.0258402541279793</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.06089684975892308</v>
+        <v>0.06089686556160453</v>
       </c>
       <c r="J2" s="1">
-        <v>0.03979398103058341</v>
+        <v>0.03979399135708812</v>
       </c>
       <c r="K2" s="1">
         <v>0</v>
@@ -25551,10 +25551,10 @@
         <v>0</v>
       </c>
       <c r="M2" s="1">
-        <v>0.08802910955250284</v>
+        <v>0.08802913239598295</v>
       </c>
       <c r="N2" s="1">
-        <v>0.03876037113368511</v>
+        <v>0.03876038119196892</v>
       </c>
       <c r="O2" s="1">
         <v>0</v>
@@ -25566,7 +25566,7 @@
         <v>0</v>
       </c>
       <c r="R2" s="1">
-        <v>0.07769301058351995</v>
+        <v>0.07769303074479104</v>
       </c>
       <c r="S2" s="1">
         <v>0</v>
@@ -25575,7 +25575,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.5279848137497902</v>
+        <v>0.5279846912622452</v>
       </c>
     </row>
     <row r="3">
@@ -25808,25 +25808,25 @@
         </is>
       </c>
       <c r="D6" s="1">
-        <v>0.09953401703587546</v>
+        <v>0.09953402737947123</v>
       </c>
       <c r="E6" s="1">
-        <v>0.08972592046664685</v>
+        <v>0.08972592979098316</v>
       </c>
       <c r="F6" s="1">
-        <v>0.02179577015384136</v>
+        <v>0.02179577241886233</v>
       </c>
       <c r="G6" s="1">
-        <v>0.1220563128615113</v>
+        <v>0.1220563255456288</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>0.07010972732818965</v>
+        <v>0.0701097346140071</v>
       </c>
       <c r="J6" s="1">
-        <v>0.01525703910768895</v>
+        <v>0.01525704069320363</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -25835,10 +25835,10 @@
         <v>0</v>
       </c>
       <c r="M6" s="1">
-        <v>0.05230984836921922</v>
+        <v>0.05230985380526955</v>
       </c>
       <c r="N6" s="1">
-        <v>0.03269365523076201</v>
+        <v>0.03269365862829347</v>
       </c>
       <c r="O6" s="1">
         <v>0</v>
@@ -25850,16 +25850,16 @@
         <v>0</v>
       </c>
       <c r="R6" s="1">
-        <v>0.0624812077743452</v>
+        <v>0.06248121426740531</v>
       </c>
       <c r="S6" s="1">
-        <v>0.01525703910768895</v>
+        <v>0.01525704069320363</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>0.4187794625642309</v>
+        <v>0.4187794021636717</v>
       </c>
     </row>
     <row r="7">
@@ -30267,16 +30267,16 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.2675326949805025</v>
+        <v>0.2675327644050124</v>
       </c>
       <c r="E2" s="1">
-        <v>0.03876037113368511</v>
+        <v>0.03876038119196892</v>
       </c>
       <c r="F2" s="1">
-        <v>0.1657221201360228</v>
+        <v>0.165722163140774</v>
       </c>
       <c r="G2" s="1">
-        <v>0.5279848137497902</v>
+        <v>0.5279846912622452</v>
       </c>
     </row>
     <row r="3">
@@ -30383,16 +30383,16 @@
         </is>
       </c>
       <c r="D6" s="1">
-        <v>0.4184787869537536</v>
+        <v>0.4184788304421563</v>
       </c>
       <c r="E6" s="1">
-        <v>0.04795069433845096</v>
+        <v>0.0479506993214971</v>
       </c>
       <c r="F6" s="1">
-        <v>0.1147910561435644</v>
+        <v>0.1147910680726749</v>
       </c>
       <c r="G6" s="1">
-        <v>0.4187794625642309</v>
+        <v>0.4187794021636717</v>
       </c>
     </row>
     <row r="7">
@@ -32322,25 +32322,25 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.1173905918896201</v>
+        <v>0.1173906043171885</v>
       </c>
       <c r="E2" s="1">
-        <v>0.05542271649464968</v>
+        <v>0.0554227223619819</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
       </c>
       <c r="G2" s="1">
-        <v>0.0316701237112284</v>
+        <v>0.03167012706398967</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.07463592487946155</v>
+        <v>0.07463593278080229</v>
       </c>
       <c r="J2" s="1">
-        <v>0.04877199051529173</v>
+        <v>0.04877199567854408</v>
       </c>
       <c r="K2" s="1">
         <v>0</v>
@@ -32349,10 +32349,10 @@
         <v>0</v>
       </c>
       <c r="M2" s="1">
-        <v>0.1078895547762516</v>
+        <v>0.1078895661979916</v>
       </c>
       <c r="N2" s="1">
-        <v>0.04750518556684256</v>
+        <v>0.04750519059598446</v>
       </c>
       <c r="O2" s="1">
         <v>0</v>
@@ -32364,7 +32364,7 @@
         <v>0</v>
       </c>
       <c r="R2" s="1">
-        <v>0.09522150529175999</v>
+        <v>0.09522151537239554</v>
       </c>
       <c r="S2" s="1">
         <v>0</v>
@@ -32373,7 +32373,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.4214924068748951</v>
+        <v>0.4214923456311226</v>
       </c>
     </row>
     <row r="3">
@@ -32606,25 +32606,25 @@
         </is>
       </c>
       <c r="D6" s="1">
-        <v>0.1353920085179377</v>
+        <v>0.1353920136897356</v>
       </c>
       <c r="E6" s="1">
-        <v>0.1220504602333234</v>
+        <v>0.1220504648954916</v>
       </c>
       <c r="F6" s="1">
-        <v>0.0296478850769207</v>
+        <v>0.02964788620943118</v>
       </c>
       <c r="G6" s="1">
-        <v>0.1660281564307555</v>
+        <v>0.1660281627728142</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>0.09536736366409483</v>
+        <v>0.09536736730700356</v>
       </c>
       <c r="J6" s="1">
-        <v>0.02075351955384449</v>
+        <v>0.02075352034660183</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -32633,10 +32633,10 @@
         <v>0</v>
       </c>
       <c r="M6" s="1">
-        <v>0.07115492418460961</v>
+        <v>0.07115492690263478</v>
       </c>
       <c r="N6" s="1">
-        <v>0.044471827615381</v>
+        <v>0.04447182931414673</v>
       </c>
       <c r="O6" s="1">
         <v>0</v>
@@ -32648,16 +32648,16 @@
         <v>0</v>
       </c>
       <c r="R6" s="1">
-        <v>0.08499060388717261</v>
+        <v>0.08499060713370268</v>
       </c>
       <c r="S6" s="1">
-        <v>0.02075351955384449</v>
+        <v>0.02075352034660183</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>0.2093897312821155</v>
+        <v>0.2093897010818359</v>
       </c>
     </row>
     <row r="7">
@@ -37065,16 +37065,16 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3278913474902515</v>
+        <v>0.3278913822025065</v>
       </c>
       <c r="E2" s="1">
-        <v>0.04750518556684256</v>
+        <v>0.04750519059598446</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2031110600680116</v>
+        <v>0.2031110815703872</v>
       </c>
       <c r="G2" s="1">
-        <v>0.4214924068748951</v>
+        <v>0.4214923456311226</v>
       </c>
     </row>
     <row r="3">
@@ -37181,16 +37181,16 @@
         </is>
       </c>
       <c r="D6" s="1">
-        <v>0.5692393934768767</v>
+        <v>0.569239415221078</v>
       </c>
       <c r="E6" s="1">
-        <v>0.0652253471692255</v>
+        <v>0.06522534966074857</v>
       </c>
       <c r="F6" s="1">
-        <v>0.1561455280717822</v>
+        <v>0.1561455340363375</v>
       </c>
       <c r="G6" s="1">
-        <v>0.2093897312821155</v>
+        <v>0.2093897010818359</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Update PDS public dashboard/state: official 2026-08, holding 2026-09
</commit_message>
<xml_diff>
--- a/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
+++ b/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
@@ -25541,28 +25541,28 @@
         </is>
       </c>
       <c r="E2" s="1">
-        <v>0.6890733242034912</v>
+        <v>0.6890734434127808</v>
       </c>
       <c r="F2" s="1">
-        <v>0.09578119206428549</v>
+        <v>0.09578120863437674</v>
       </c>
       <c r="G2" s="1">
-        <v>0.04522043690085413</v>
+        <v>0.04522044472396376</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.02584024965763094</v>
+        <v>0.0258402541279793</v>
       </c>
       <c r="J2" s="1">
         <v>0</v>
       </c>
       <c r="K2" s="1">
-        <v>0.06089685502648356</v>
+        <v>0.06089686556160453</v>
       </c>
       <c r="L2" s="1">
-        <v>0.03979398447275164</v>
+        <v>0.03979399135708812</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -25571,10 +25571,10 @@
         <v>0</v>
       </c>
       <c r="O2" s="1">
-        <v>0.08802911716699621</v>
+        <v>0.08802913239598295</v>
       </c>
       <c r="P2" s="1">
-        <v>0.03876037448644638</v>
+        <v>0.03876038119196892</v>
       </c>
       <c r="Q2" s="1">
         <v>0</v>
@@ -25586,7 +25586,7 @@
         <v>0</v>
       </c>
       <c r="T2" s="1">
-        <v>0.07769301730394365</v>
+        <v>0.07769303074479104</v>
       </c>
       <c r="U2" s="1">
         <v>0</v>
@@ -25595,7 +25595,7 @@
         <v>0</v>
       </c>
       <c r="W2" s="1">
-        <v>0.5279847729206085</v>
+        <v>0.5279846912622452</v>
       </c>
     </row>
     <row r="3">
@@ -25857,28 +25857,28 @@
         </is>
       </c>
       <c r="E6" s="1">
-        <v>0.5812205444138646</v>
+        <v>0.581220639074136</v>
       </c>
       <c r="F6" s="1">
-        <v>0.09953401823087432</v>
+        <v>0.0995340344414458</v>
       </c>
       <c r="G6" s="1">
-        <v>0.08972592154389034</v>
+        <v>0.08972593615706974</v>
       </c>
       <c r="H6" s="1">
-        <v>0.02179577041551994</v>
+        <v>0.02179577396528012</v>
       </c>
       <c r="I6" s="1">
-        <v>0.1220563143269114</v>
+        <v>0.1220563342055684</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
       </c>
       <c r="K6" s="1">
-        <v>0.07010972816992242</v>
+        <v>0.07010973958831766</v>
       </c>
       <c r="L6" s="1">
-        <v>0.01525703929086396</v>
+        <v>0.01525704177569609</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -25887,10 +25887,10 @@
         <v>0</v>
       </c>
       <c r="O6" s="1">
-        <v>0.05230984899724782</v>
+        <v>0.05230985751667225</v>
       </c>
       <c r="P6" s="1">
-        <v>0.03269365562327989</v>
+        <v>0.03269366094792015</v>
       </c>
       <c r="Q6" s="1">
         <v>0</v>
@@ -25902,16 +25902,16 @@
         <v>0</v>
       </c>
       <c r="T6" s="1">
-        <v>0.06248120852449047</v>
+        <v>0.06248121870046965</v>
       </c>
       <c r="U6" s="1">
-        <v>0.01525703929086396</v>
+        <v>0.01525704177569609</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>0.4187794555861354</v>
+        <v>0.418779360925864</v>
       </c>
     </row>
     <row r="7">
@@ -30824,19 +30824,19 @@
         </is>
       </c>
       <c r="E2" s="1">
-        <v>0.6890733242034912</v>
+        <v>0.6890734434127808</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2675327181220057</v>
+        <v>0.2675327644050124</v>
       </c>
       <c r="G2" s="1">
-        <v>0.03876037448644638</v>
+        <v>0.03876038119196892</v>
       </c>
       <c r="H2" s="1">
-        <v>0.1657221344709399</v>
+        <v>0.165722163140774</v>
       </c>
       <c r="I2" s="1">
-        <v>0.5279847729206085</v>
+        <v>0.5279846912622452</v>
       </c>
     </row>
     <row r="3">
@@ -30972,19 +30972,19 @@
         </is>
       </c>
       <c r="E6" s="1">
-        <v>0.5812205444138646</v>
+        <v>0.581220639074136</v>
       </c>
       <c r="F6" s="1">
-        <v>0.4184787919779824</v>
+        <v>0.4184788601333778</v>
       </c>
       <c r="G6" s="1">
-        <v>0.04795069491414385</v>
+        <v>0.04795070272361624</v>
       </c>
       <c r="H6" s="1">
-        <v>0.1147910575217383</v>
+        <v>0.1147910762171419</v>
       </c>
       <c r="I6" s="1">
-        <v>0.4187794555861354</v>
+        <v>0.418779360925864</v>
       </c>
     </row>
     <row r="7">
@@ -33402,25 +33402,25 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.1173905960321429</v>
+        <v>0.1173906043171885</v>
       </c>
       <c r="E2" s="1">
-        <v>0.05542271845042708</v>
+        <v>0.0554227223619819</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
       </c>
       <c r="G2" s="1">
-        <v>0.03167012482881549</v>
+        <v>0.03167012706398967</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.0746359275132418</v>
+        <v>0.07463593278080229</v>
       </c>
       <c r="J2" s="1">
-        <v>0.04877199223637584</v>
+        <v>0.04877199567854408</v>
       </c>
       <c r="K2" s="1">
         <v>0</v>
@@ -33429,10 +33429,10 @@
         <v>0</v>
       </c>
       <c r="M2" s="1">
-        <v>0.1078895585834983</v>
+        <v>0.1078895661979916</v>
       </c>
       <c r="N2" s="1">
-        <v>0.0475051872432232</v>
+        <v>0.04750519059598446</v>
       </c>
       <c r="O2" s="1">
         <v>0</v>
@@ -33444,7 +33444,7 @@
         <v>0</v>
       </c>
       <c r="R2" s="1">
-        <v>0.09522150865197183</v>
+        <v>0.09522151537239554</v>
       </c>
       <c r="S2" s="1">
         <v>0</v>
@@ -33453,7 +33453,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.4214923864603043</v>
+        <v>0.4214923456311226</v>
       </c>
     </row>
     <row r="3">
@@ -33686,25 +33686,25 @@
         </is>
       </c>
       <c r="D6" s="1">
-        <v>0.1353920091154372</v>
+        <v>0.1353920172207229</v>
       </c>
       <c r="E6" s="1">
-        <v>0.1220504607719452</v>
+        <v>0.1220504680785349</v>
       </c>
       <c r="F6" s="1">
-        <v>0.02964788520775999</v>
+        <v>0.02964788698264008</v>
       </c>
       <c r="G6" s="1">
-        <v>0.1660281571634556</v>
+        <v>0.1660281671027841</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>0.09536736408496121</v>
+        <v>0.09536736979415883</v>
       </c>
       <c r="J6" s="1">
-        <v>0.020753519645432</v>
+        <v>0.02075352088784806</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -33713,10 +33713,10 @@
         <v>0</v>
       </c>
       <c r="M6" s="1">
-        <v>0.07115492449862391</v>
+        <v>0.07115492875833612</v>
       </c>
       <c r="N6" s="1">
-        <v>0.04447182781163994</v>
+        <v>0.04447183047396008</v>
       </c>
       <c r="O6" s="1">
         <v>0</v>
@@ -33728,16 +33728,16 @@
         <v>0</v>
       </c>
       <c r="R6" s="1">
-        <v>0.08499060426224525</v>
+        <v>0.08499060935023484</v>
       </c>
       <c r="S6" s="1">
-        <v>0.020753519645432</v>
+        <v>0.02075352088784806</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>0.2093897277930677</v>
+        <v>0.209389680462932</v>
       </c>
     </row>
     <row r="7">
@@ -38145,16 +38145,16 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3278913590610031</v>
+        <v>0.3278913822025065</v>
       </c>
       <c r="E2" s="1">
-        <v>0.0475051872432232</v>
+        <v>0.04750519059598446</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2031110672354701</v>
+        <v>0.2031110815703872</v>
       </c>
       <c r="G2" s="1">
-        <v>0.4214923864603043</v>
+        <v>0.4214923456311226</v>
       </c>
     </row>
     <row r="3">
@@ -38261,16 +38261,16 @@
         </is>
       </c>
       <c r="D6" s="1">
-        <v>0.5692393959889912</v>
+        <v>0.5692394300666889</v>
       </c>
       <c r="E6" s="1">
-        <v>0.06522534745707194</v>
+        <v>0.06522535136180814</v>
       </c>
       <c r="F6" s="1">
-        <v>0.1561455287608692</v>
+        <v>0.156145538108571</v>
       </c>
       <c r="G6" s="1">
-        <v>0.2093897277930677</v>
+        <v>0.209389680462932</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Update PDS public dashboard/state: official 2026-09, holding 2026-10
</commit_message>
<xml_diff>
--- a/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
+++ b/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
@@ -25422,7 +25422,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREVIEW</t>
+          <t xml:space="preserve">OFFICIAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -25441,28 +25441,28 @@
         </is>
       </c>
       <c r="E2" s="1">
-        <v>0.730446457862854</v>
+        <v>0.7122377157211304</v>
       </c>
       <c r="F2" s="1">
-        <v>0.07852299422025684</v>
+        <v>0.09526179447770097</v>
       </c>
       <c r="G2" s="1">
-        <v>0.04793554879724982</v>
+        <v>0.0467406000941992</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.02739174216985705</v>
+        <v>0.02670891433954241</v>
       </c>
       <c r="J2" s="1">
         <v>0</v>
       </c>
       <c r="K2" s="1">
-        <v>0.07030547156929971</v>
+        <v>0.05920476011931895</v>
       </c>
       <c r="L2" s="1">
-        <v>0.04793554879724982</v>
+        <v>0.03739248007535932</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -25471,10 +25471,10 @@
         <v>0</v>
       </c>
       <c r="O2" s="1">
-        <v>0.09906680084764979</v>
+        <v>0.06944317728281001</v>
       </c>
       <c r="P2" s="1">
-        <v>0.04108761325478554</v>
+        <v>0.04006337150931358</v>
       </c>
       <c r="Q2" s="1">
         <v>0</v>
@@ -25483,10 +25483,10 @@
         <v>0</v>
       </c>
       <c r="S2" s="1">
-        <v>0.02876132927834988</v>
+        <v>0.01780594289302826</v>
       </c>
       <c r="T2" s="1">
-        <v>0.05934877470135689</v>
+        <v>0.05786931440234185</v>
       </c>
       <c r="U2" s="1">
         <v>0</v>
@@ -25495,7 +25495,7 @@
         <v>0</v>
       </c>
       <c r="W2" s="1">
-        <v>0.499644176363945</v>
+        <v>0.5495096448063848</v>
       </c>
     </row>
     <row r="3">
@@ -25757,28 +25757,28 @@
         </is>
       </c>
       <c r="E6" s="1">
-        <v>0.5812204769124886</v>
+        <v>0.5812205304998401</v>
       </c>
       <c r="F6" s="1">
-        <v>0.09953400667126368</v>
+        <v>0.09953401584809762</v>
       </c>
       <c r="G6" s="1">
-        <v>0.08972591112336542</v>
+        <v>0.0897259193959128</v>
       </c>
       <c r="H6" s="1">
-        <v>0.02179576788421834</v>
+        <v>0.02179576989374402</v>
       </c>
       <c r="I6" s="1">
-        <v>0.1220563001516224</v>
+        <v>0.1220563114049663</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
       </c>
       <c r="K6" s="1">
-        <v>0.07010972002756893</v>
+        <v>0.07010972649154322</v>
       </c>
       <c r="L6" s="1">
-        <v>0.01525703751895284</v>
+        <v>0.01525703892562082</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -25787,10 +25787,10 @@
         <v>0</v>
       </c>
       <c r="O6" s="1">
-        <v>0.05230984292212398</v>
+        <v>0.05230984774498561</v>
       </c>
       <c r="P6" s="1">
-        <v>0.03269365182632748</v>
+        <v>0.03269365484061601</v>
       </c>
       <c r="Q6" s="1">
         <v>0</v>
@@ -25802,16 +25802,16 @@
         <v>0</v>
       </c>
       <c r="T6" s="1">
-        <v>0.06248120126809254</v>
+        <v>0.06248120702873284</v>
       </c>
       <c r="U6" s="1">
-        <v>0.01525703751895284</v>
+        <v>0.01525703892562082</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>0.4187795230875114</v>
+        <v>0.4187794695001599</v>
       </c>
     </row>
     <row r="7">
@@ -30705,7 +30705,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREVIEW</t>
+          <t xml:space="preserve">OFFICIAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -30724,19 +30724,19 @@
         </is>
       </c>
       <c r="E2" s="1">
-        <v>0.730446457862854</v>
+        <v>0.7122377157211304</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2720913055539132</v>
+        <v>0.2653085491061208</v>
       </c>
       <c r="G2" s="1">
-        <v>0.04108761325478554</v>
+        <v>0.04006337150931358</v>
       </c>
       <c r="H2" s="1">
-        <v>0.1871769048273565</v>
+        <v>0.1451184345781801</v>
       </c>
       <c r="I2" s="1">
-        <v>0.499644176363945</v>
+        <v>0.5495096448063848</v>
       </c>
     </row>
     <row r="3">
@@ -30872,19 +30872,19 @@
         </is>
       </c>
       <c r="E6" s="1">
-        <v>0.5812204769124886</v>
+        <v>0.5812205304998401</v>
       </c>
       <c r="F6" s="1">
-        <v>0.4184787433769916</v>
+        <v>0.4184787819598847</v>
       </c>
       <c r="G6" s="1">
-        <v>0.04795068934528032</v>
+        <v>0.04795069376623683</v>
       </c>
       <c r="H6" s="1">
-        <v>0.1147910441902165</v>
+        <v>0.1147910547737185</v>
       </c>
       <c r="I6" s="1">
-        <v>0.4187795230875114</v>
+        <v>0.4187794695001599</v>
       </c>
     </row>
     <row r="7">
@@ -33515,25 +33515,25 @@
         </is>
       </c>
       <c r="D5" s="1">
-        <v>0.1353920033356318</v>
+        <v>0.1353920079240488</v>
       </c>
       <c r="E5" s="1">
-        <v>0.1220504555616827</v>
+        <v>0.1220504596979564</v>
       </c>
       <c r="F5" s="1">
-        <v>0.02964788394210919</v>
+        <v>0.02964788494687203</v>
       </c>
       <c r="G5" s="1">
-        <v>0.1660281500758111</v>
+        <v>0.166028155702483</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>0.09536736001378447</v>
+        <v>0.09536736324577161</v>
       </c>
       <c r="J5" s="1">
-        <v>0.02075351875947644</v>
+        <v>0.02075351946281043</v>
       </c>
       <c r="K5" s="1">
         <v>0</v>
@@ -33542,10 +33542,10 @@
         <v>0</v>
       </c>
       <c r="M5" s="1">
-        <v>0.07115492146106199</v>
+        <v>0.07115492387249281</v>
       </c>
       <c r="N5" s="1">
-        <v>0.04447182591316375</v>
+        <v>0.044471827420308</v>
       </c>
       <c r="O5" s="1">
         <v>0</v>
@@ -33557,16 +33557,16 @@
         <v>0</v>
       </c>
       <c r="R5" s="1">
-        <v>0.08499060063404629</v>
+        <v>0.08499060351436644</v>
       </c>
       <c r="S5" s="1">
-        <v>0.02075351875947644</v>
+        <v>0.02075351946281043</v>
       </c>
       <c r="T5" s="1">
         <v>0</v>
       </c>
       <c r="U5" s="1">
-        <v>0.2093897615437557</v>
+        <v>0.2093897347500799</v>
       </c>
     </row>
     <row r="6">
@@ -38061,16 +38061,16 @@
         </is>
       </c>
       <c r="D5" s="1">
-        <v>0.5692393716884957</v>
+        <v>0.5692393909799423</v>
       </c>
       <c r="E5" s="1">
-        <v>0.06522534467264018</v>
+        <v>0.06522534688311843</v>
       </c>
       <c r="F5" s="1">
-        <v>0.1561455220951083</v>
+        <v>0.1561455273868592</v>
       </c>
       <c r="G5" s="1">
-        <v>0.2093897615437557</v>
+        <v>0.2093897347500799</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Stage reviewed PDS hosted artifacts (not released)
</commit_message>
<xml_diff>
--- a/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
+++ b/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
@@ -229,10 +229,10 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="E2" s="1">
-        <v>0.06562500000000003</v>
+        <v>0.09187499999999971</v>
       </c>
       <c r="F2" s="1">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="G2" s="1">
         <v>0.03750000000000003</v>
@@ -265,7 +265,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="R2" s="1">
         <v>0.05625</v>
@@ -277,7 +277,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -18175,16 +18175,16 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3462499999999998</v>
+        <v>0.3974999999999995</v>
       </c>
       <c r="E2" s="1">
         <v>0.05625</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2037499999999997</v>
+        <v>0.1787499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -25647,10 +25647,10 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.06562500000000003</v>
+        <v>0.09187499999999971</v>
       </c>
       <c r="H2" s="1">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="I2" s="1">
         <v>0.03750000000000003</v>
@@ -25683,7 +25683,7 @@
         <v>0</v>
       </c>
       <c r="S2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="T2" s="1">
         <v>0.05625</v>
@@ -25695,7 +25695,7 @@
         <v>0</v>
       </c>
       <c r="W2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -26036,28 +26036,28 @@
         </is>
       </c>
       <c r="E7" s="1">
-        <v>0.5812205392093202</v>
+        <v>0.5812205928018681</v>
       </c>
       <c r="F7" s="1">
-        <v>0.09953401733959609</v>
+        <v>0.09953402651731992</v>
       </c>
       <c r="G7" s="1">
-        <v>0.08972592074043879</v>
+        <v>0.08972592901378838</v>
       </c>
       <c r="H7" s="1">
-        <v>0.02179577022034953</v>
+        <v>0.02179577223007007</v>
       </c>
       <c r="I7" s="1">
-        <v>0.1220563132339571</v>
+        <v>0.1220563244883921</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>0.07010972754212424</v>
+        <v>0.07010973400672535</v>
       </c>
       <c r="L7" s="1">
-        <v>0.01525703915424467</v>
+        <v>0.01525704056104906</v>
       </c>
       <c r="M7" s="1">
         <v>0</v>
@@ -26066,10 +26066,10 @@
         <v>0</v>
       </c>
       <c r="O7" s="1">
-        <v>0.05230984852883882</v>
+        <v>0.05230985335216814</v>
       </c>
       <c r="P7" s="1">
-        <v>0.03269365533052426</v>
+        <v>0.03269365834510508</v>
       </c>
       <c r="Q7" s="1">
         <v>0</v>
@@ -26081,16 +26081,16 @@
         <v>0</v>
       </c>
       <c r="T7" s="1">
-        <v>0.06248120796500194</v>
+        <v>0.06248121372620084</v>
       </c>
       <c r="U7" s="1">
-        <v>0.01525703915424467</v>
+        <v>0.01525704056104906</v>
       </c>
       <c r="V7" s="1">
         <v>0</v>
       </c>
       <c r="W7" s="1">
-        <v>0.4187794607906798</v>
+        <v>0.4187794071981319</v>
       </c>
     </row>
     <row r="8">
@@ -31006,16 +31006,16 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>0.3462499999999998</v>
+        <v>0.3974999999999995</v>
       </c>
       <c r="G2" s="1">
         <v>0.05625</v>
       </c>
       <c r="H2" s="1">
-        <v>0.2037499999999997</v>
+        <v>0.1787499999999997</v>
       </c>
       <c r="I2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -31188,19 +31188,19 @@
         </is>
       </c>
       <c r="E7" s="1">
-        <v>0.5812205392093202</v>
+        <v>0.5812205928018681</v>
       </c>
       <c r="F7" s="1">
-        <v>0.4184787882307104</v>
+        <v>0.4184788268173449</v>
       </c>
       <c r="G7" s="1">
-        <v>0.04795069448476894</v>
+        <v>0.04795069890615414</v>
       </c>
       <c r="H7" s="1">
-        <v>0.1147910564938407</v>
+        <v>0.114791067078369</v>
       </c>
       <c r="I7" s="1">
-        <v>0.4187794607906798</v>
+        <v>0.4187794071981319</v>
       </c>
     </row>
     <row r="8">
@@ -33621,10 +33621,10 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="E2" s="1">
-        <v>0.06562500000000003</v>
+        <v>0.09187499999999971</v>
       </c>
       <c r="F2" s="1">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="G2" s="1">
         <v>0.03750000000000003</v>
@@ -33657,7 +33657,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="R2" s="1">
         <v>0.05625</v>
@@ -33669,7 +33669,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -33973,25 +33973,25 @@
         </is>
       </c>
       <c r="D7" s="1">
-        <v>0.1353920086697981</v>
+        <v>0.13539201325866</v>
       </c>
       <c r="E7" s="1">
-        <v>0.1220504603702194</v>
+        <v>0.1220504645068942</v>
       </c>
       <c r="F7" s="1">
-        <v>0.02964788511017478</v>
+        <v>0.02964788611503505</v>
       </c>
       <c r="G7" s="1">
-        <v>0.1660281566169784</v>
+        <v>0.1660281622441959</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>0.09536736377106213</v>
+        <v>0.09536736700336268</v>
       </c>
       <c r="J7" s="1">
-        <v>0.02075351957712235</v>
+        <v>0.02075352028052454</v>
       </c>
       <c r="K7" s="1">
         <v>0</v>
@@ -34000,10 +34000,10 @@
         <v>0</v>
       </c>
       <c r="M7" s="1">
-        <v>0.07115492426441941</v>
+        <v>0.07115492667608407</v>
       </c>
       <c r="N7" s="1">
-        <v>0.04447182766526213</v>
+        <v>0.04447182917255255</v>
       </c>
       <c r="O7" s="1">
         <v>0</v>
@@ -34015,16 +34015,16 @@
         <v>0</v>
       </c>
       <c r="R7" s="1">
-        <v>0.084990603982501</v>
+        <v>0.08499060686310045</v>
       </c>
       <c r="S7" s="1">
-        <v>0.02075351957712235</v>
+        <v>0.02075352028052454</v>
       </c>
       <c r="T7" s="1">
         <v>0</v>
       </c>
       <c r="U7" s="1">
-        <v>0.2093897303953399</v>
+        <v>0.2093897035990659</v>
       </c>
     </row>
     <row r="8">
@@ -38432,16 +38432,16 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3462499999999998</v>
+        <v>0.3974999999999995</v>
       </c>
       <c r="E2" s="1">
         <v>0.05625</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2037499999999997</v>
+        <v>0.1787499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -38577,16 +38577,16 @@
         </is>
       </c>
       <c r="D7" s="1">
-        <v>0.5692393941153551</v>
+        <v>0.5692394134086723</v>
       </c>
       <c r="E7" s="1">
-        <v>0.06522534724238448</v>
+        <v>0.06522534945307709</v>
       </c>
       <c r="F7" s="1">
-        <v>0.1561455282469204</v>
+        <v>0.1561455335391845</v>
       </c>
       <c r="G7" s="1">
-        <v>0.2093897303953399</v>
+        <v>0.2093897035990659</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Publish reviewed PDS 2026-10-09 hosted intake snapshot
Source audited hosted candidate SHA256 b898e3c913f8e75c630da951b4be6197f1a503d155304f0e27d6d28f3b511548. PRICEVINT-001 bounded historical return restatement: internal reviewed exception accepted by owner. Spot FX is noncanonical sensitivity, not forward/NDF live P&L. Preserve local Windows operational publish path until changed-live parity is verified.
</commit_message>
<xml_diff>
--- a/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
+++ b/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
@@ -229,10 +229,10 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="E2" s="1">
-        <v>0.06562500000000003</v>
+        <v>0.09187499999999971</v>
       </c>
       <c r="F2" s="1">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="G2" s="1">
         <v>0.03750000000000003</v>
@@ -265,7 +265,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="R2" s="1">
         <v>0.05625</v>
@@ -277,7 +277,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -18175,16 +18175,16 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3462499999999998</v>
+        <v>0.3974999999999995</v>
       </c>
       <c r="E2" s="1">
         <v>0.05625</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2037499999999997</v>
+        <v>0.1787499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -25647,10 +25647,10 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.06562500000000003</v>
+        <v>0.09187499999999971</v>
       </c>
       <c r="H2" s="1">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="I2" s="1">
         <v>0.03750000000000003</v>
@@ -25683,7 +25683,7 @@
         <v>0</v>
       </c>
       <c r="S2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="T2" s="1">
         <v>0.05625</v>
@@ -25695,7 +25695,7 @@
         <v>0</v>
       </c>
       <c r="W2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -26036,28 +26036,28 @@
         </is>
       </c>
       <c r="E7" s="1">
-        <v>0.5812205392093202</v>
+        <v>0.5812205928018681</v>
       </c>
       <c r="F7" s="1">
-        <v>0.09953401733959609</v>
+        <v>0.09953402651731992</v>
       </c>
       <c r="G7" s="1">
-        <v>0.08972592074043879</v>
+        <v>0.08972592901378838</v>
       </c>
       <c r="H7" s="1">
-        <v>0.02179577022034953</v>
+        <v>0.02179577223007007</v>
       </c>
       <c r="I7" s="1">
-        <v>0.1220563132339571</v>
+        <v>0.1220563244883921</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>0.07010972754212424</v>
+        <v>0.07010973400672535</v>
       </c>
       <c r="L7" s="1">
-        <v>0.01525703915424467</v>
+        <v>0.01525704056104906</v>
       </c>
       <c r="M7" s="1">
         <v>0</v>
@@ -26066,10 +26066,10 @@
         <v>0</v>
       </c>
       <c r="O7" s="1">
-        <v>0.05230984852883882</v>
+        <v>0.05230985335216814</v>
       </c>
       <c r="P7" s="1">
-        <v>0.03269365533052426</v>
+        <v>0.03269365834510508</v>
       </c>
       <c r="Q7" s="1">
         <v>0</v>
@@ -26081,16 +26081,16 @@
         <v>0</v>
       </c>
       <c r="T7" s="1">
-        <v>0.06248120796500194</v>
+        <v>0.06248121372620084</v>
       </c>
       <c r="U7" s="1">
-        <v>0.01525703915424467</v>
+        <v>0.01525704056104906</v>
       </c>
       <c r="V7" s="1">
         <v>0</v>
       </c>
       <c r="W7" s="1">
-        <v>0.4187794607906798</v>
+        <v>0.4187794071981319</v>
       </c>
     </row>
     <row r="8">
@@ -31006,16 +31006,16 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>0.3462499999999998</v>
+        <v>0.3974999999999995</v>
       </c>
       <c r="G2" s="1">
         <v>0.05625</v>
       </c>
       <c r="H2" s="1">
-        <v>0.2037499999999997</v>
+        <v>0.1787499999999997</v>
       </c>
       <c r="I2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -31188,19 +31188,19 @@
         </is>
       </c>
       <c r="E7" s="1">
-        <v>0.5812205392093202</v>
+        <v>0.5812205928018681</v>
       </c>
       <c r="F7" s="1">
-        <v>0.4184787882307104</v>
+        <v>0.4184788268173449</v>
       </c>
       <c r="G7" s="1">
-        <v>0.04795069448476894</v>
+        <v>0.04795069890615414</v>
       </c>
       <c r="H7" s="1">
-        <v>0.1147910564938407</v>
+        <v>0.114791067078369</v>
       </c>
       <c r="I7" s="1">
-        <v>0.4187794607906798</v>
+        <v>0.4187794071981319</v>
       </c>
     </row>
     <row r="8">
@@ -33621,10 +33621,10 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="E2" s="1">
-        <v>0.06562500000000003</v>
+        <v>0.09187499999999971</v>
       </c>
       <c r="F2" s="1">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="G2" s="1">
         <v>0.03750000000000003</v>
@@ -33657,7 +33657,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="R2" s="1">
         <v>0.05625</v>
@@ -33669,7 +33669,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -33973,25 +33973,25 @@
         </is>
       </c>
       <c r="D7" s="1">
-        <v>0.1353920086697981</v>
+        <v>0.13539201325866</v>
       </c>
       <c r="E7" s="1">
-        <v>0.1220504603702194</v>
+        <v>0.1220504645068942</v>
       </c>
       <c r="F7" s="1">
-        <v>0.02964788511017478</v>
+        <v>0.02964788611503505</v>
       </c>
       <c r="G7" s="1">
-        <v>0.1660281566169784</v>
+        <v>0.1660281622441959</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>0.09536736377106213</v>
+        <v>0.09536736700336268</v>
       </c>
       <c r="J7" s="1">
-        <v>0.02075351957712235</v>
+        <v>0.02075352028052454</v>
       </c>
       <c r="K7" s="1">
         <v>0</v>
@@ -34000,10 +34000,10 @@
         <v>0</v>
       </c>
       <c r="M7" s="1">
-        <v>0.07115492426441941</v>
+        <v>0.07115492667608407</v>
       </c>
       <c r="N7" s="1">
-        <v>0.04447182766526213</v>
+        <v>0.04447182917255255</v>
       </c>
       <c r="O7" s="1">
         <v>0</v>
@@ -34015,16 +34015,16 @@
         <v>0</v>
       </c>
       <c r="R7" s="1">
-        <v>0.084990603982501</v>
+        <v>0.08499060686310045</v>
       </c>
       <c r="S7" s="1">
-        <v>0.02075351957712235</v>
+        <v>0.02075352028052454</v>
       </c>
       <c r="T7" s="1">
         <v>0</v>
       </c>
       <c r="U7" s="1">
-        <v>0.2093897303953399</v>
+        <v>0.2093897035990659</v>
       </c>
     </row>
     <row r="8">
@@ -38432,16 +38432,16 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3462499999999998</v>
+        <v>0.3974999999999995</v>
       </c>
       <c r="E2" s="1">
         <v>0.05625</v>
       </c>
       <c r="F2" s="1">
-        <v>0.2037499999999997</v>
+        <v>0.1787499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.39375</v>
+        <v>0.3674999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -38577,16 +38577,16 @@
         </is>
       </c>
       <c r="D7" s="1">
-        <v>0.5692393941153551</v>
+        <v>0.5692394134086723</v>
       </c>
       <c r="E7" s="1">
-        <v>0.06522534724238448</v>
+        <v>0.06522534945307709</v>
       </c>
       <c r="F7" s="1">
-        <v>0.1561455282469204</v>
+        <v>0.1561455335391845</v>
       </c>
       <c r="G7" s="1">
-        <v>0.2093897303953399</v>
+        <v>0.2093897035990659</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Publish reviewed PDS refresh through 2026-10-14
Reviewed PDS hosted intake PR #26. Approved publication of the exact 19-file source snapshot and derived platform bindings. Official signal 2026-09, holding 2026-10, market-through 2026-10-14; source vintage review restricted to this candidate.
</commit_message>
<xml_diff>
--- a/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
+++ b/public/assets/systems/pds/PDS_Portfolio_History_Current_Definition.xlsx
@@ -229,19 +229,19 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="E2" s="1">
-        <v>0.09187499999999971</v>
+        <v>0.1168749999999997</v>
       </c>
       <c r="F2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="G2" s="1">
-        <v>0.03750000000000003</v>
+        <v>0.01125</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.08312499999999998</v>
+        <v>0.030625</v>
       </c>
       <c r="J2" s="1">
         <v>0.02625000000000003</v>
@@ -277,7 +277,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.3674999999999997</v>
+        <v>0.4462499999999997</v>
       </c>
     </row>
     <row r="3">
@@ -18175,7 +18175,7 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3974999999999995</v>
+        <v>0.3187499999999995</v>
       </c>
       <c r="E2" s="1">
         <v>0.05625</v>
@@ -18184,7 +18184,7 @@
         <v>0.1787499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.3674999999999997</v>
+        <v>0.4462499999999997</v>
       </c>
     </row>
     <row r="3">
@@ -25647,19 +25647,19 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.09187499999999971</v>
+        <v>0.1168749999999997</v>
       </c>
       <c r="H2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.03750000000000003</v>
+        <v>0.01125</v>
       </c>
       <c r="J2" s="1">
         <v>0</v>
       </c>
       <c r="K2" s="1">
-        <v>0.08312499999999998</v>
+        <v>0.030625</v>
       </c>
       <c r="L2" s="1">
         <v>0.02625000000000003</v>
@@ -25695,7 +25695,7 @@
         <v>0</v>
       </c>
       <c r="W2" s="1">
-        <v>0.3674999999999997</v>
+        <v>0.4462499999999997</v>
       </c>
     </row>
     <row r="3">
@@ -26036,28 +26036,28 @@
         </is>
       </c>
       <c r="E7" s="1">
-        <v>0.5812205042632564</v>
+        <v>0.5812204586440203</v>
       </c>
       <c r="F7" s="1">
-        <v>0.09953401135508268</v>
+        <v>0.09953400354278848</v>
       </c>
       <c r="G7" s="1">
-        <v>0.0897259153456402</v>
+        <v>0.08972590830317062</v>
       </c>
       <c r="H7" s="1">
-        <v>0.02179576890987214</v>
+        <v>0.02179576719915078</v>
       </c>
       <c r="I7" s="1">
-        <v>0.1220563058952837</v>
+        <v>0.1220562963152441</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>0.07010972332675532</v>
+        <v>0.07010971782393495</v>
       </c>
       <c r="L7" s="1">
-        <v>0.0152570382369105</v>
+        <v>0.01525703703940555</v>
       </c>
       <c r="M7" s="1">
         <v>0</v>
@@ -26066,10 +26066,10 @@
         <v>0</v>
       </c>
       <c r="O7" s="1">
-        <v>0.05230984538369308</v>
+        <v>0.05230984127796183</v>
       </c>
       <c r="P7" s="1">
-        <v>0.03269365336480817</v>
+        <v>0.03269365079872614</v>
       </c>
       <c r="Q7" s="1">
         <v>0</v>
@@ -26081,16 +26081,16 @@
         <v>0</v>
       </c>
       <c r="T7" s="1">
-        <v>0.06248120420830009</v>
+        <v>0.0624811993042322</v>
       </c>
       <c r="U7" s="1">
-        <v>0.0152570382369105</v>
+        <v>0.01525703703940555</v>
       </c>
       <c r="V7" s="1">
         <v>0</v>
       </c>
       <c r="W7" s="1">
-        <v>0.4187794957367436</v>
+        <v>0.4187795413559797</v>
       </c>
     </row>
     <row r="8">
@@ -31006,7 +31006,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>0.3974999999999995</v>
+        <v>0.3187499999999995</v>
       </c>
       <c r="G2" s="1">
         <v>0.05625</v>
@@ -31015,7 +31015,7 @@
         <v>0.1787499999999997</v>
       </c>
       <c r="I2" s="1">
-        <v>0.3674999999999997</v>
+        <v>0.4462499999999997</v>
       </c>
     </row>
     <row r="3">
@@ -31188,19 +31188,19 @@
         </is>
       </c>
       <c r="E7" s="1">
-        <v>0.5812205042632564</v>
+        <v>0.5812204586440203</v>
       </c>
       <c r="F7" s="1">
-        <v>0.4184787630695445</v>
+        <v>0.4184787302236945</v>
       </c>
       <c r="G7" s="1">
-        <v>0.04795069160171867</v>
+        <v>0.04795068783813169</v>
       </c>
       <c r="H7" s="1">
-        <v>0.1147910495919932</v>
+        <v>0.114791040582194</v>
       </c>
       <c r="I7" s="1">
-        <v>0.4187794957367436</v>
+        <v>0.4187795413559797</v>
       </c>
     </row>
     <row r="8">
@@ -33621,19 +33621,19 @@
         <v>0.1337499999999997</v>
       </c>
       <c r="E2" s="1">
-        <v>0.09187499999999971</v>
+        <v>0.1168749999999997</v>
       </c>
       <c r="F2" s="1">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="G2" s="1">
-        <v>0.03750000000000003</v>
+        <v>0.01125</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
       </c>
       <c r="I2" s="1">
-        <v>0.08312499999999998</v>
+        <v>0.030625</v>
       </c>
       <c r="J2" s="1">
         <v>0.02625000000000003</v>
@@ -33669,7 +33669,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.3674999999999997</v>
+        <v>0.4462499999999997</v>
       </c>
     </row>
     <row r="3">
@@ -33973,25 +33973,25 @@
         </is>
       </c>
       <c r="D7" s="1">
-        <v>0.1353920056775413</v>
+        <v>0.1353920017713942</v>
       </c>
       <c r="E7" s="1">
-        <v>0.1220504576728201</v>
+        <v>0.1220504541515853</v>
       </c>
       <c r="F7" s="1">
-        <v>0.02964788445493608</v>
+        <v>0.02964788359957541</v>
       </c>
       <c r="G7" s="1">
-        <v>0.1660281529476417</v>
+        <v>0.1660281481576219</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>0.09536736166337767</v>
+        <v>0.09536735891196749</v>
       </c>
       <c r="J7" s="1">
-        <v>0.02075351911845526</v>
+        <v>0.02075351851970279</v>
       </c>
       <c r="K7" s="1">
         <v>0</v>
@@ -34000,10 +34000,10 @@
         <v>0</v>
       </c>
       <c r="M7" s="1">
-        <v>0.07115492269184655</v>
+        <v>0.07115492063898092</v>
       </c>
       <c r="N7" s="1">
-        <v>0.04447182668240408</v>
+        <v>0.04447182539936307</v>
       </c>
       <c r="O7" s="1">
         <v>0</v>
@@ -34015,16 +34015,16 @@
         <v>0</v>
       </c>
       <c r="R7" s="1">
-        <v>0.08499060210415006</v>
+        <v>0.08499059965211612</v>
       </c>
       <c r="S7" s="1">
-        <v>0.02075351911845526</v>
+        <v>0.02075351851970279</v>
       </c>
       <c r="T7" s="1">
         <v>0</v>
       </c>
       <c r="U7" s="1">
-        <v>0.2093897478683718</v>
+        <v>0.2093897706779899</v>
       </c>
     </row>
     <row r="8">
@@ -38432,7 +38432,7 @@
         </is>
       </c>
       <c r="D2" s="1">
-        <v>0.3974999999999995</v>
+        <v>0.3187499999999995</v>
       </c>
       <c r="E2" s="1">
         <v>0.05625</v>
@@ -38441,7 +38441,7 @@
         <v>0.1787499999999997</v>
       </c>
       <c r="G2" s="1">
-        <v>0.3674999999999997</v>
+        <v>0.4462499999999997</v>
       </c>
     </row>
     <row r="3">
@@ -38577,16 +38577,16 @@
         </is>
       </c>
       <c r="D7" s="1">
-        <v>0.5692393815347722</v>
+        <v>0.5692393651118471</v>
       </c>
       <c r="E7" s="1">
-        <v>0.06522534580085934</v>
+        <v>0.06522534391906586</v>
       </c>
       <c r="F7" s="1">
-        <v>0.1561455247959966</v>
+        <v>0.156145520291097</v>
       </c>
       <c r="G7" s="1">
-        <v>0.2093897478683718</v>
+        <v>0.2093897706779899</v>
       </c>
     </row>
     <row r="8">

</xml_diff>